<commit_message>
Show current cycle only, allow notes on current or latest cycle and update Limhjul steps
</commit_message>
<xml_diff>
--- a/Limhjul.xlsx
+++ b/Limhjul.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedometic-my.sharepoint.com/personal/martin_petersson_dometic_com/Documents/Apps/steps&amp;times/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{7E9D086A-D70A-4A3E-9BAC-6067635BFF5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6A7300C-C75E-47CB-98C6-840ED6F5F1CB}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{7E9D086A-D70A-4A3E-9BAC-6067635BFF5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4111D770-B6B2-4F3F-AEDD-CE528E1529C4}"/>
   <bookViews>
-    <workbookView xWindow="42000" yWindow="2580" windowWidth="28800" windowHeight="15345" xr2:uid="{4F768552-8E62-44F9-B993-09B113426101}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{4F768552-8E62-44F9-B993-09B113426101}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Steg</t>
   </si>
@@ -47,22 +47,19 @@
     <t>Moment</t>
   </si>
   <si>
-    <t>Hämta material</t>
-  </si>
-  <si>
-    <t>Placera på bord</t>
-  </si>
-  <si>
-    <t>Sätt på ettikett/distans</t>
-  </si>
-  <si>
     <t>Rengör material</t>
   </si>
   <si>
-    <t>Ladda maskin</t>
-  </si>
-  <si>
     <t>Placera material i vagn</t>
+  </si>
+  <si>
+    <t>Hämta material och placera på bord</t>
+  </si>
+  <si>
+    <t>Dra folie och sätt på ettikett/distans</t>
+  </si>
+  <si>
+    <t>Ladda/lossa maskin</t>
   </si>
 </sst>
 </file>
@@ -146,8 +143,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{95D404B6-BA61-486C-BE40-ACC559512E1A}" name="Tabell1" displayName="Tabell1" ref="A1:B7" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B7" xr:uid="{42258919-B15B-41E8-BD41-FA7CA9D6CB91}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{95D404B6-BA61-486C-BE40-ACC559512E1A}" name="Tabell1" displayName="Tabell1" ref="A1:B6" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B6" xr:uid="{42258919-B15B-41E8-BD41-FA7CA9D6CB91}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{23ECBC60-ED4D-46B9-828B-EBE9769B3DAC}" name="Steg"/>
     <tableColumn id="2" xr3:uid="{433925F9-5D6B-4BE3-B771-370E7A3381DA}" name="Moment"/>
@@ -473,10 +470,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7286161-B96E-4403-AE94-C9FFAD901A05}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -492,47 +489,39 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>